<commit_message>
[auto-snapshot] 2026-04-26 16:00 | onda-hompage | 57 files
</commit_message>
<xml_diff>
--- a/naver-place-crawler/results_health/분당_헬스장.xlsx
+++ b/naver-place-crawler/results_health/분당_헬스장.xlsx
@@ -417,22 +417,22 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V11"/>
+  <dimension ref="A1:V19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="21" customWidth="1" min="2" max="2"/>
-    <col width="27" customWidth="1" min="3" max="3"/>
+    <col width="31" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
     <col width="10" customWidth="1" min="6" max="6"/>
-    <col width="37" customWidth="1" min="7" max="7"/>
+    <col width="47" customWidth="1" min="7" max="7"/>
     <col width="50" customWidth="1" min="8" max="8"/>
     <col width="10" customWidth="1" min="9" max="9"/>
     <col width="10" customWidth="1" min="10" max="10"/>
     <col width="10" customWidth="1" min="11" max="11"/>
     <col width="10" customWidth="1" min="12" max="12"/>
-    <col width="35" customWidth="1" min="13" max="13"/>
+    <col width="10" customWidth="1" min="13" max="13"/>
     <col width="10" customWidth="1" min="14" max="14"/>
     <col width="10" customWidth="1" min="15" max="15"/>
     <col width="10" customWidth="1" min="16" max="16"/>
@@ -564,29 +564,29 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>자마이카피트니스 분당정자점</t>
+          <t>필립발리휘트니스 정자본점</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>jamaica_jeongja@naver.com</t>
+          <t>ballydesign@naver.com</t>
         </is>
       </c>
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
-          <t>0507-1383-8533</t>
+          <t>031-728-7771</t>
         </is>
       </c>
       <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr">
         <is>
-          <t>경기 성남시 분당구 정자일로 121 지하 1층</t>
+          <t>경기도 성남시 분당구 내정로 58</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/jamaica_bundang?igsh=MWY4cGIybjlodW11bw%3D%3D&amp;utm_source=qr</t>
+          <t>https://blog.naver.com/ballydesign</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -601,19 +601,15 @@
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>O</t>
-        </is>
-      </c>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>https://talk.naver.com/ct/wsknjve</t>
-        </is>
-      </c>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr"/>
       <c r="N2" t="inlineStr">
         <is>
           <t>X</t>
@@ -625,13 +621,13 @@
         </is>
       </c>
       <c r="P2" t="n">
-        <v>1841</v>
+        <v>237</v>
       </c>
       <c r="Q2" t="n">
-        <v>223</v>
+        <v>94</v>
       </c>
       <c r="R2" t="n">
-        <v>2064</v>
+        <v>331</v>
       </c>
       <c r="S2" t="inlineStr">
         <is>
@@ -640,12 +636,12 @@
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>1710539074</t>
+          <t>158436174</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
         <is>
-          <t>https://m.place.naver.com/place/1710539074</t>
+          <t>https://m.place.naver.com/place/158436174</t>
         </is>
       </c>
       <c r="V2" t="inlineStr">
@@ -662,34 +658,34 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>뉴핏휘트니스 정자점</t>
+          <t>비전휘트니스 분당점</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>newfit_csj@naver.com</t>
+          <t>visionfitness555@naver.com</t>
         </is>
       </c>
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
-          <t>0507-1347-6714</t>
+          <t>0507-1439-8755</t>
         </is>
       </c>
       <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr">
         <is>
-          <t>경기 성남시 분당구 정자로76번길 11 한라프라자</t>
+          <t>경기도 성남시 분당구 돌마로 46 광천프라자 2층</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/newfit_csj</t>
+          <t>https://litt.ly/visionfitness05</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
@@ -699,19 +695,15 @@
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>X</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>O</t>
-        </is>
-      </c>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t>https://talk.naver.com/ct/w4k06n</t>
-        </is>
-      </c>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr"/>
       <c r="N3" t="inlineStr">
         <is>
           <t>X</t>
@@ -723,13 +715,13 @@
         </is>
       </c>
       <c r="P3" t="n">
-        <v>1137</v>
+        <v>2471</v>
       </c>
       <c r="Q3" t="n">
-        <v>966</v>
+        <v>1919</v>
       </c>
       <c r="R3" t="n">
-        <v>2103</v>
+        <v>4390</v>
       </c>
       <c r="S3" t="inlineStr">
         <is>
@@ -738,12 +730,12 @@
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>36782451</t>
+          <t>1765794431</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
         <is>
-          <t>https://m.place.naver.com/place/36782451</t>
+          <t>https://m.place.naver.com/place/1765794431</t>
         </is>
       </c>
       <c r="V3" t="inlineStr">
@@ -760,29 +752,29 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>스포짐 판교점</t>
+          <t>자마이카피트니스 분당정자점</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>spogym_2@naver.com</t>
+          <t>jamaica_jeongja@naver.com</t>
         </is>
       </c>
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
-          <t>0507-1476-8384</t>
+          <t>0507-1383-8533</t>
         </is>
       </c>
       <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr">
         <is>
-          <t>경기 성남시 분당구 대왕판교로 670 유스페이스2 B동 지하1층</t>
+          <t>경기도 성남시 분당구 정자일로 121 지하 1층</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/spogym_pg</t>
+          <t>https://www.instagram.com/jamaica_bundang?igsh=MWY4cGIybjlodW11bw%3D%3D&amp;utm_source=qr</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -802,14 +794,10 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>O</t>
-        </is>
-      </c>
-      <c r="M4" t="inlineStr">
-        <is>
-          <t>https://talk.naver.com/ct/wpasubw</t>
-        </is>
-      </c>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr"/>
       <c r="N4" t="inlineStr">
         <is>
           <t>X</t>
@@ -821,13 +809,13 @@
         </is>
       </c>
       <c r="P4" t="n">
-        <v>731</v>
+        <v>1841</v>
       </c>
       <c r="Q4" t="n">
-        <v>624</v>
+        <v>223</v>
       </c>
       <c r="R4" t="n">
-        <v>1355</v>
+        <v>2064</v>
       </c>
       <c r="S4" t="inlineStr">
         <is>
@@ -836,12 +824,12 @@
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>20123697</t>
+          <t>1710539074</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
         <is>
-          <t>https://m.place.naver.com/place/20123697</t>
+          <t>https://m.place.naver.com/place/1710539074</t>
         </is>
       </c>
       <c r="V4" t="inlineStr">
@@ -858,29 +846,29 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>스포애니 야탑역점</t>
+          <t>그라운드피트니스</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>spoany90@naver.com</t>
+          <t>ground-fitness@naver.com</t>
         </is>
       </c>
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
-          <t>0507-1337-9618</t>
+          <t>0507-1464-5758</t>
         </is>
       </c>
       <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr">
         <is>
-          <t>경기 성남시 분당구 성남대로 926 메트로빌딩 8층</t>
+          <t>경기도 성남시 분당구 서현로 170 풍림아이원플러스 3층 301호</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>http://m.spoany.co.kr/branch/branch_detail.html?base_seq=MTA1</t>
+          <t>https://blog.naver.com/ground-fitness</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
@@ -895,19 +883,15 @@
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>O</t>
-        </is>
-      </c>
-      <c r="M5" t="inlineStr">
-        <is>
-          <t>https://talk.naver.com/ct/w5il7f</t>
-        </is>
-      </c>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr"/>
       <c r="N5" t="inlineStr">
         <is>
           <t>X</t>
@@ -919,13 +903,13 @@
         </is>
       </c>
       <c r="P5" t="n">
-        <v>706</v>
+        <v>374</v>
       </c>
       <c r="Q5" t="n">
-        <v>1494</v>
+        <v>1211</v>
       </c>
       <c r="R5" t="n">
-        <v>2200</v>
+        <v>1585</v>
       </c>
       <c r="S5" t="inlineStr">
         <is>
@@ -934,12 +918,12 @@
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>1115298912</t>
+          <t>1472483345</t>
         </is>
       </c>
       <c r="U5" t="inlineStr">
         <is>
-          <t>https://m.place.naver.com/place/1115298912</t>
+          <t>https://m.place.naver.com/place/1472483345</t>
         </is>
       </c>
       <c r="V5" t="inlineStr">
@@ -956,30 +940,34 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>뭉트니스 야탑</t>
+          <t>익스홀릭 가넷 야탑점</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>mtns1@naver.com</t>
+          <t>exholic-yatop@naver.com</t>
         </is>
       </c>
       <c r="D6" t="inlineStr"/>
-      <c r="E6" t="inlineStr"/>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>0507-1486-1557</t>
+        </is>
+      </c>
       <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr">
         <is>
-          <t>경기 성남시 분당구 장미로 55 장미마을 지하1층</t>
+          <t>경기도 성남시 분당구 야탑로 95 세신옴니코아빌딩</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/mtns_leader</t>
+          <t>http://익스홀릭가넷야탑점.shop/</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
@@ -1009,13 +997,13 @@
         </is>
       </c>
       <c r="P6" t="n">
-        <v>284</v>
+        <v>1960</v>
       </c>
       <c r="Q6" t="n">
-        <v>1036</v>
+        <v>1273</v>
       </c>
       <c r="R6" t="n">
-        <v>1320</v>
+        <v>3233</v>
       </c>
       <c r="S6" t="inlineStr">
         <is>
@@ -1024,12 +1012,12 @@
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>1657314482</t>
+          <t>13581227</t>
         </is>
       </c>
       <c r="U6" t="inlineStr">
         <is>
-          <t>https://m.place.naver.com/place/1657314482</t>
+          <t>https://m.place.naver.com/place/13581227</t>
         </is>
       </c>
       <c r="V6" t="inlineStr">
@@ -1046,29 +1034,29 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>헬스보이짐&amp;필라걸&amp;골프인 분당정자점</t>
+          <t>업투 분당서현점</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>healthboy90_@naver.com</t>
+          <t>uptofitness5@naver.com</t>
         </is>
       </c>
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
-          <t>0507-1419-2436</t>
+          <t>0507-1346-5229</t>
         </is>
       </c>
       <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr">
         <is>
-          <t>경기 성남시 분당구 성남대로331번길 13 7층 701-706호</t>
+          <t>경기도 성남시 분당구 중앙공원로40번길 8 현대근린상가 지하1층 5호</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/healthboy90_/223799590825</t>
+          <t>https://www.instagram.com/upto_seohyun/</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
@@ -1083,19 +1071,15 @@
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>X</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>O</t>
-        </is>
-      </c>
-      <c r="M7" t="inlineStr">
-        <is>
-          <t>https://talk.naver.com/ct/wli4sqi</t>
-        </is>
-      </c>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr"/>
       <c r="N7" t="inlineStr">
         <is>
           <t>X</t>
@@ -1107,13 +1091,13 @@
         </is>
       </c>
       <c r="P7" t="n">
-        <v>457</v>
+        <v>1157</v>
       </c>
       <c r="Q7" t="n">
-        <v>751</v>
+        <v>723</v>
       </c>
       <c r="R7" t="n">
-        <v>1208</v>
+        <v>1880</v>
       </c>
       <c r="S7" t="inlineStr">
         <is>
@@ -1122,12 +1106,12 @@
       </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>1989525945</t>
+          <t>1984136642</t>
         </is>
       </c>
       <c r="U7" t="inlineStr">
         <is>
-          <t>https://m.place.naver.com/place/1989525945</t>
+          <t>https://m.place.naver.com/place/1984136642</t>
         </is>
       </c>
       <c r="V7" t="inlineStr">
@@ -1139,34 +1123,34 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>스포츠시설</t>
+          <t>헬스장</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>헬스보이짐 헬스 PT 판교역점</t>
+          <t>크로스핏 테디짐 분당</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>healthboygym78@naver.com</t>
+          <t>cftdg@naver.com</t>
         </is>
       </c>
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
-          <t>0507-1402-1275</t>
+          <t>0507-1365-1447</t>
         </is>
       </c>
       <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr">
         <is>
-          <t>경기 성남시 분당구 대왕판교로606번길 58 지하1층</t>
+          <t>경기도 성남시 분당구 정자일로198번길 15 지하1층</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/healthboygym78/223380215625</t>
+          <t>https://www.instagram.com/teddygym</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
@@ -1181,22 +1165,18 @@
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>X</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>O</t>
-        </is>
-      </c>
-      <c r="M8" t="inlineStr">
-        <is>
-          <t>https://talk.naver.com/ct/wi2wapb</t>
-        </is>
-      </c>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr"/>
       <c r="N8" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
@@ -1205,13 +1185,13 @@
         </is>
       </c>
       <c r="P8" t="n">
-        <v>2540</v>
+        <v>395</v>
       </c>
       <c r="Q8" t="n">
-        <v>323</v>
+        <v>79</v>
       </c>
       <c r="R8" t="n">
-        <v>2863</v>
+        <v>474</v>
       </c>
       <c r="S8" t="inlineStr">
         <is>
@@ -1220,12 +1200,12 @@
       </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t>1835201778</t>
+          <t>36406982</t>
         </is>
       </c>
       <c r="U8" t="inlineStr">
         <is>
-          <t>https://m.place.naver.com/place/1835201778</t>
+          <t>https://m.place.naver.com/place/36406982</t>
         </is>
       </c>
       <c r="V8" t="inlineStr">
@@ -1242,29 +1222,29 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>익스홀릭 가넷 미금점</t>
+          <t>밥스짐 분당점</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>dydwk147@naver.com</t>
+          <t>ish0674@naver.com</t>
         </is>
       </c>
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
-          <t>0507-1429-2557</t>
+          <t>0507-1474-7017</t>
         </is>
       </c>
       <c r="F9" t="inlineStr"/>
       <c r="G9" t="inlineStr">
         <is>
-          <t>경기 성남시 분당구 돌마로 87 골드프라자 6층 가넷휘트니스</t>
+          <t>경기도 성남시 분당구 성남대로 449 로얄팰리스 에이동 212, 213, 214호</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/dydwk147</t>
+          <t>https://www.instagram.com/bobsgymbob/profilecard/?igsh=MTFxcDRvanRsZ2ZyNA==</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
@@ -1279,19 +1259,15 @@
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>X</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>O</t>
-        </is>
-      </c>
-      <c r="M9" t="inlineStr">
-        <is>
-          <t>https://talk.naver.com/ct/w4n5lk</t>
-        </is>
-      </c>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr"/>
       <c r="N9" t="inlineStr">
         <is>
           <t>X</t>
@@ -1303,13 +1279,13 @@
         </is>
       </c>
       <c r="P9" t="n">
-        <v>561</v>
+        <v>82</v>
       </c>
       <c r="Q9" t="n">
-        <v>1074</v>
+        <v>185</v>
       </c>
       <c r="R9" t="n">
-        <v>1635</v>
+        <v>267</v>
       </c>
       <c r="S9" t="inlineStr">
         <is>
@@ -1318,12 +1294,12 @@
       </c>
       <c r="T9" t="inlineStr">
         <is>
-          <t>12763227</t>
+          <t>1581057750</t>
         </is>
       </c>
       <c r="U9" t="inlineStr">
         <is>
-          <t>https://m.place.naver.com/place/12763227</t>
+          <t>https://m.place.naver.com/place/1581057750</t>
         </is>
       </c>
       <c r="V9" t="inlineStr">
@@ -1340,34 +1316,34 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>런던피트니스&amp;필라테스 분당이매점</t>
+          <t>투엑스휘트니스 분당점</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>londoner83@naver.com</t>
+          <t>2xfit@naver.com</t>
         </is>
       </c>
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr">
         <is>
-          <t>0507-1406-9679</t>
+          <t>031-782-5115</t>
         </is>
       </c>
       <c r="F10" t="inlineStr"/>
       <c r="G10" t="inlineStr">
         <is>
-          <t>경기 성남시 분당구 성남대로779번길 13 오성프라자빌딩 5층</t>
+          <t>경기도 성남시 분당구 정자일로 177 분당인텔리지2 3F</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/londoner83</t>
+          <t>http://www.2xfitness.co.kr/</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
@@ -1382,14 +1358,10 @@
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>O</t>
-        </is>
-      </c>
-      <c r="M10" t="inlineStr">
-        <is>
-          <t>https://talk.naver.com/ct/w4pnpp</t>
-        </is>
-      </c>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr"/>
       <c r="N10" t="inlineStr">
         <is>
           <t>X</t>
@@ -1401,13 +1373,13 @@
         </is>
       </c>
       <c r="P10" t="n">
-        <v>1340</v>
+        <v>431</v>
       </c>
       <c r="Q10" t="n">
-        <v>473</v>
+        <v>28</v>
       </c>
       <c r="R10" t="n">
-        <v>1813</v>
+        <v>459</v>
       </c>
       <c r="S10" t="inlineStr">
         <is>
@@ -1416,12 +1388,12 @@
       </c>
       <c r="T10" t="inlineStr">
         <is>
-          <t>13530251</t>
+          <t>32278618</t>
         </is>
       </c>
       <c r="U10" t="inlineStr">
         <is>
-          <t>https://m.place.naver.com/place/13530251</t>
+          <t>https://m.place.naver.com/place/32278618</t>
         </is>
       </c>
       <c r="V10" t="inlineStr">
@@ -1438,29 +1410,29 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>험블 휘트니스 PT</t>
+          <t>헬스보이짐 헬스 PT 판교역점</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>humblefitness@naver.com</t>
+          <t>healthboygym78@naver.com</t>
         </is>
       </c>
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr">
         <is>
-          <t>031-697-8768</t>
+          <t>0507-1402-1275</t>
         </is>
       </c>
       <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr">
         <is>
-          <t>경기 성남시 분당구 성남대로331번길 3-3 701호</t>
+          <t>경기도 성남시 분당구 대왕판교로606번길 58 지하1층</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/humblefitness</t>
+          <t>https://blog.naver.com/healthboygym78/223380215625</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
@@ -1480,14 +1452,10 @@
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>O</t>
-        </is>
-      </c>
-      <c r="M11" t="inlineStr">
-        <is>
-          <t>https://talk.naver.com/ct/wnvkt3b</t>
-        </is>
-      </c>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr"/>
       <c r="N11" t="inlineStr">
         <is>
           <t>X</t>
@@ -1499,13 +1467,13 @@
         </is>
       </c>
       <c r="P11" t="n">
-        <v>141</v>
+        <v>2540</v>
       </c>
       <c r="Q11" t="n">
-        <v>1437</v>
+        <v>323</v>
       </c>
       <c r="R11" t="n">
-        <v>1578</v>
+        <v>2863</v>
       </c>
       <c r="S11" t="inlineStr">
         <is>
@@ -1514,15 +1482,767 @@
       </c>
       <c r="T11" t="inlineStr">
         <is>
-          <t>1134171602</t>
+          <t>1835201778</t>
         </is>
       </c>
       <c r="U11" t="inlineStr">
         <is>
-          <t>https://m.place.naver.com/place/1134171602</t>
+          <t>https://m.place.naver.com/place/1835201778</t>
         </is>
       </c>
       <c r="V11" t="inlineStr">
+        <is>
+          <t>2026-04-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>헬스장</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>엔엘휘트니스 분당이매점</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>nlfitness2@naver.com</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr"/>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>0507-1415-2075</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr"/>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>경기도 성남시 분당구 판교로 440 지하1층</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/nlfitness2_imae/</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr"/>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="P12" t="n">
+        <v>642</v>
+      </c>
+      <c r="Q12" t="n">
+        <v>241</v>
+      </c>
+      <c r="R12" t="n">
+        <v>883</v>
+      </c>
+      <c r="S12" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="T12" t="inlineStr">
+        <is>
+          <t>1194690742</t>
+        </is>
+      </c>
+      <c r="U12" t="inlineStr">
+        <is>
+          <t>https://m.place.naver.com/place/1194690742</t>
+        </is>
+      </c>
+      <c r="V12" t="inlineStr">
+        <is>
+          <t>2026-04-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>스포츠시설</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>헬스보이짐&amp;필라걸 수내점</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>healthboy40@naver.com</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr"/>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>0507-1380-2239</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr"/>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>경기도 성남시 분당구 내정로173번길 49 5층</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>https://blog.naver.com/healthboy40/223688037867</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr"/>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="P13" t="n">
+        <v>968</v>
+      </c>
+      <c r="Q13" t="n">
+        <v>734</v>
+      </c>
+      <c r="R13" t="n">
+        <v>1702</v>
+      </c>
+      <c r="S13" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="T13" t="inlineStr">
+        <is>
+          <t>1973151166</t>
+        </is>
+      </c>
+      <c r="U13" t="inlineStr">
+        <is>
+          <t>https://m.place.naver.com/place/1973151166</t>
+        </is>
+      </c>
+      <c r="V13" t="inlineStr">
+        <is>
+          <t>2026-04-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>헬스장</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>헤일로짐24시 헬스 PT 판교점</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>halogym02@naver.com</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr"/>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>0507-1315-8840</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr"/>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>경기도 성남시 분당구 대왕판교로 660 유스페이스1 지하1층 127호</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>https://booking.naver.com/booking/6/bizes/933331</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M14" t="inlineStr"/>
+      <c r="N14" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="O14" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="P14" t="n">
+        <v>663</v>
+      </c>
+      <c r="Q14" t="n">
+        <v>929</v>
+      </c>
+      <c r="R14" t="n">
+        <v>1592</v>
+      </c>
+      <c r="S14" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="T14" t="inlineStr">
+        <is>
+          <t>1806695299</t>
+        </is>
+      </c>
+      <c r="U14" t="inlineStr">
+        <is>
+          <t>https://m.place.naver.com/place/1806695299</t>
+        </is>
+      </c>
+      <c r="V14" t="inlineStr">
+        <is>
+          <t>2026-04-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>헬스장</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>피트니스비엠 분당 서현점</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>ksk2023@naver.com</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr"/>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>0507-1443-0942</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr"/>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>경기도 성남시 분당구 돌마로 482 주영빌딩 지하 1층</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/fitnessbm._.hyoja</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M15" t="inlineStr"/>
+      <c r="N15" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="O15" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="P15" t="n">
+        <v>513</v>
+      </c>
+      <c r="Q15" t="n">
+        <v>684</v>
+      </c>
+      <c r="R15" t="n">
+        <v>1197</v>
+      </c>
+      <c r="S15" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="T15" t="inlineStr">
+        <is>
+          <t>36333115</t>
+        </is>
+      </c>
+      <c r="U15" t="inlineStr">
+        <is>
+          <t>https://m.place.naver.com/place/36333115</t>
+        </is>
+      </c>
+      <c r="V15" t="inlineStr">
+        <is>
+          <t>2026-04-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>스포츠시설</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>베러댄 휘트니스 분당야탑점</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>56zqrwcwsv@naver.com</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr"/>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>0507-1438-9698</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr"/>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>경기도 성남시 분당구 야탑로75번길 15 세화빌딩 4층</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>https://blog.naver.com/56zqrwcwsv</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr"/>
+      <c r="N16" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="O16" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="P16" t="n">
+        <v>382</v>
+      </c>
+      <c r="Q16" t="n">
+        <v>2085</v>
+      </c>
+      <c r="R16" t="n">
+        <v>2467</v>
+      </c>
+      <c r="S16" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="T16" t="inlineStr">
+        <is>
+          <t>1013682807</t>
+        </is>
+      </c>
+      <c r="U16" t="inlineStr">
+        <is>
+          <t>https://m.place.naver.com/place/1013682807</t>
+        </is>
+      </c>
+      <c r="V16" t="inlineStr">
+        <is>
+          <t>2026-04-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>스포츠시설</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>쓰리핏PT 분당정자점</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>3fits@naver.com</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr"/>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>0507-1409-3559</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr"/>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>경기도 성남시 분당구 내정로113번길 4 2층 202호, 203-1호</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>https://3fitpt.com</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr"/>
+      <c r="N17" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="O17" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="P17" t="n">
+        <v>357</v>
+      </c>
+      <c r="Q17" t="n">
+        <v>800</v>
+      </c>
+      <c r="R17" t="n">
+        <v>1157</v>
+      </c>
+      <c r="S17" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="T17" t="inlineStr">
+        <is>
+          <t>1845673431</t>
+        </is>
+      </c>
+      <c r="U17" t="inlineStr">
+        <is>
+          <t>https://m.place.naver.com/place/1845673431</t>
+        </is>
+      </c>
+      <c r="V17" t="inlineStr">
+        <is>
+          <t>2026-04-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>스포츠시설</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>밀라노짐 수내점</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>milanos_1@naver.com</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr"/>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>0507-1335-9682</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr"/>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>경기도 성남시 분당구 내정로166번길 5 원전빌딩 B1층</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>http://www.instagram.com/milanogym_s</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M18" t="inlineStr"/>
+      <c r="N18" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="O18" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="P18" t="n">
+        <v>1141</v>
+      </c>
+      <c r="Q18" t="n">
+        <v>696</v>
+      </c>
+      <c r="R18" t="n">
+        <v>1837</v>
+      </c>
+      <c r="S18" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="T18" t="inlineStr">
+        <is>
+          <t>1843911670</t>
+        </is>
+      </c>
+      <c r="U18" t="inlineStr">
+        <is>
+          <t>https://m.place.naver.com/place/1843911670</t>
+        </is>
+      </c>
+      <c r="V18" t="inlineStr">
+        <is>
+          <t>2026-04-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>스포츠시설</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>비율라이프 바디코치 여성전용 체형필라테스 PT 야탑점</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>rockrock1256@naver.com</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr"/>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>0507-1445-2430</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr"/>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>경기도 성남시 분당구 야탑로69번길 8 2층 바디코치 야탑점</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/official_bodycoach?igsh=MTF6cmlnd240MTdwMg%3D%3D&amp;utm_source=qr</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M19" t="inlineStr"/>
+      <c r="N19" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="O19" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="P19" t="n">
+        <v>203</v>
+      </c>
+      <c r="Q19" t="n">
+        <v>786</v>
+      </c>
+      <c r="R19" t="n">
+        <v>989</v>
+      </c>
+      <c r="S19" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="T19" t="inlineStr">
+        <is>
+          <t>1723811790</t>
+        </is>
+      </c>
+      <c r="U19" t="inlineStr">
+        <is>
+          <t>https://m.place.naver.com/place/1723811790</t>
+        </is>
+      </c>
+      <c r="V19" t="inlineStr">
         <is>
           <t>2026-04-26</t>
         </is>

</xml_diff>